<commit_message>
Correct Week 2 timesheet dates
</commit_message>
<xml_diff>
--- a/ShijianZhu_S394861/Week_2/timesheet_ShijianZhu_S394861.xlsx
+++ b/ShijianZhu_S394861/Week_2/timesheet_ShijianZhu_S394861.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 2" sheetId="1" r:id="R3f71634b5fe74cc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 2" sheetId="1" r:id="R6ec7e04c08074403"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -549,7 +549,7 @@
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="40" t="n">
-        <x:v>46237</x:v>
+        <x:v>46230</x:v>
       </x:c>
       <x:c r="B7" s="41" t="n">
         <x:v>1</x:v>
@@ -569,7 +569,7 @@
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="40" t="n">
-        <x:v>46237</x:v>
+        <x:v>46230</x:v>
       </x:c>
       <x:c r="B8" s="41" t="n">
         <x:v>2</x:v>
@@ -589,7 +589,7 @@
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="40" t="n">
-        <x:v>46237</x:v>
+        <x:v>46230</x:v>
       </x:c>
       <x:c r="B9" s="41" t="n">
         <x:v>3</x:v>
@@ -609,7 +609,7 @@
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="40" t="n">
-        <x:v>46238</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="B10" s="41" t="n">
         <x:v>4</x:v>
@@ -629,7 +629,7 @@
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="40" t="n">
-        <x:v>46238</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="B11" s="41" t="n">
         <x:v>5</x:v>
@@ -649,7 +649,7 @@
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="40" t="n">
-        <x:v>46238</x:v>
+        <x:v>46231</x:v>
       </x:c>
       <x:c r="B12" s="41" t="n">
         <x:v>6</x:v>
@@ -669,7 +669,7 @@
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="40" t="n">
-        <x:v>46239</x:v>
+        <x:v>46232</x:v>
       </x:c>
       <x:c r="B13" s="41" t="n">
         <x:v>7</x:v>
@@ -689,7 +689,7 @@
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="40" t="n">
-        <x:v>46239</x:v>
+        <x:v>46232</x:v>
       </x:c>
       <x:c r="B14" s="41" t="n">
         <x:v>8</x:v>
@@ -709,7 +709,7 @@
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="40" t="n">
-        <x:v>46239</x:v>
+        <x:v>46232</x:v>
       </x:c>
       <x:c r="B15" s="41" t="n">
         <x:v>9</x:v>
@@ -729,7 +729,7 @@
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
       <x:c r="A16" s="40" t="n">
-        <x:v>46240</x:v>
+        <x:v>46233</x:v>
       </x:c>
       <x:c r="B16" s="41" t="n">
         <x:v>10</x:v>
@@ -749,7 +749,7 @@
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="40" t="n">
-        <x:v>46240</x:v>
+        <x:v>46233</x:v>
       </x:c>
       <x:c r="B17" s="41" t="n">
         <x:v>11</x:v>
@@ -769,7 +769,7 @@
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
       <x:c r="A18" s="40" t="n">
-        <x:v>46240</x:v>
+        <x:v>46233</x:v>
       </x:c>
       <x:c r="B18" s="41" t="n">
         <x:v>12</x:v>
@@ -789,7 +789,7 @@
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
       <x:c r="A19" s="40" t="n">
-        <x:v>46241</x:v>
+        <x:v>46234</x:v>
       </x:c>
       <x:c r="B19" s="41" t="n">
         <x:v>13</x:v>
@@ -809,7 +809,7 @@
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="40" t="n">
-        <x:v>46241</x:v>
+        <x:v>46234</x:v>
       </x:c>
       <x:c r="B20" s="41" t="n">
         <x:v>14</x:v>
@@ -829,7 +829,7 @@
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
       <x:c r="A21" s="40" t="n">
-        <x:v>46241</x:v>
+        <x:v>46234</x:v>
       </x:c>
       <x:c r="B21" s="41" t="n">
         <x:v>15</x:v>
@@ -849,7 +849,7 @@
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
       <x:c r="A22" s="40" t="n">
-        <x:v>46242</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="B22" s="41" t="n">
         <x:v>16</x:v>
@@ -869,7 +869,7 @@
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="40" t="n">
-        <x:v>46242</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="B23" s="41" t="n">
         <x:v>17</x:v>
@@ -889,7 +889,7 @@
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
       <x:c r="A24" s="40" t="n">
-        <x:v>46242</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="B24" s="41" t="n">
         <x:v>18</x:v>
@@ -909,7 +909,7 @@
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
       <x:c r="A25" s="40" t="n">
-        <x:v>46243</x:v>
+        <x:v>46236</x:v>
       </x:c>
       <x:c r="B25" s="41" t="n">
         <x:v>19</x:v>
@@ -929,7 +929,7 @@
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
       <x:c r="A26" s="45" t="n">
-        <x:v>46243</x:v>
+        <x:v>46236</x:v>
       </x:c>
       <x:c r="B26" s="46" t="n">
         <x:v>20</x:v>
@@ -956,7 +956,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ddf0a07972f4c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R260a54e8247440a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>